<commit_message>
feat: Add settings sheet for map center and zoom
</commit_message>
<xml_diff>
--- a/sample_map_data.xlsx
+++ b/sample_map_data.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jiaweiqi/Documents/GitHub/assignment-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C574AB67-0E2B-DF4D-8F14-4B89D9F20431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28EE5C29-E364-CC42-93F4-574481D0D7AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17800" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="markers" sheetId="1" r:id="rId1"/>
     <sheet name="lines" sheetId="2" r:id="rId2"/>
-    <sheet name="polygons" sheetId="3" r:id="rId3"/>
-    <sheet name="heatmap" sheetId="4" r:id="rId4"/>
-    <sheet name="circles" sheetId="5" r:id="rId5"/>
+    <sheet name="settings" sheetId="6" r:id="rId3"/>
+    <sheet name="polygons" sheetId="3" r:id="rId4"/>
+    <sheet name="heatmap" sheetId="4" r:id="rId5"/>
+    <sheet name="circles" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="61">
   <si>
     <t>latitude</t>
   </si>
@@ -198,6 +199,15 @@
   </si>
   <si>
     <t>[[25.7984,-80.2027],[25.7950,-80.2867]]</t>
+  </si>
+  <si>
+    <t>center_lat</t>
+  </si>
+  <si>
+    <t>center_lon</t>
+  </si>
+  <si>
+    <t>zoom_start</t>
   </si>
 </sst>
 </file>
@@ -245,9 +255,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -776,6 +789,38 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14EB83F4-9358-4F4A-9479-CC5DE459162F}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2">
+        <v>25.796700000000001</v>
+      </c>
+      <c r="B2" s="2">
+        <v>-80.244699999999995</v>
+      </c>
+      <c r="C2" s="2">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -854,7 +899,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -1429,7 +1474,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>